<commit_message>
Load Invictus auction bid data (15 franchises, 102 players)
Replace placeholder teams/examples with the real auction data: rename the
15 teams to their franchise names, populate all 102 bought players with
their winning bids, and rename team sheet tabs to match. Verified every
team's computed spend against the source 'Total Amount Spent' totals.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JPS2A9PhrR4uvRcvaVtGkU
</commit_message>
<xml_diff>
--- a/Cricket_Auction_Tracker.xlsx
+++ b/Cricket_Auction_Tracker.xlsx
@@ -9,21 +9,21 @@
   <sheets>
     <sheet name="Auction" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Balance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Team 1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Team 2" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Team 3" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Team 4" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Team 5" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Team 6" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Team 7" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Team 8" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Team 9" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Team 10" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Team 11" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Team 12" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Team 13" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Team 14" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Team 15" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Mumbai Indians" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Royal Challangers Banglore" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Chennai Super Kings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Kolkata Knight Riders" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Patna Panthers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Sunrisers Hydrabad" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Delhi Capitals" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gujarat Titans" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Lucknow Super Giants" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Imphal Igniter" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Punjab Kings" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Rising Pune Super Giants" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Rajasthan Royals" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Kochi Tuskers" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Guwahati Chargers" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -613,15 +613,15 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Player_X</t>
+          <t>Rohit Sharma</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>2</v>
+        <v>26.5</v>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Team 4</t>
+          <t>Mumbai Indians</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -637,547 +637,1517 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Rohit S.</t>
+          <t>Kartik Tyagi</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>3.5</v>
+        <v>12</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Mumbai Indians</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Bumrah</t>
+          <t>Kuldeep Yadav</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>4.2</v>
+        <v>20</v>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Team 4</t>
+          <t>Mumbai Indians</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Kohli</t>
+          <t>Hugh Weibgen</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Team 7</t>
+          <t>Mumbai Indians</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Jadeja</t>
+          <t>Matthew Potts</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>1.2</v>
+        <v>5</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Mumbai Indians</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="11" t="n"/>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Chamika Karunaratne</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Mumbai Indians</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="7" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Karun Nair</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Mumbai Indians</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="11" t="n"/>
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Sachin Baby</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Mumbai Indians</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="7" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Anrich Nortje</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Mumbai Indians</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="11" t="n"/>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Navdeep Saini</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="7" t="n"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Harnoor Singh</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="11" t="n"/>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Swastik Chikara</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="7" t="n"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Tilak Varma</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="11" t="n"/>
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Dawid Malan</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="7" t="n"/>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Haris Rauf</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="11" t="n"/>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>George Scrimshaw</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="7" t="n"/>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Hasan Ali</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="11" t="n"/>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Usma Mir</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="7" t="n"/>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Jimmy Neesham</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="n"/>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="11" t="n"/>
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Parth Rekhade</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n"/>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="7" t="n"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Dinesh Bana</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="n"/>
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="11" t="n"/>
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Yuzvendra Chahal</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Royal Challangers Banglore</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n"/>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="7" t="n"/>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Sandeep Sharma</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="n"/>
-      <c r="B28" s="10" t="n"/>
-      <c r="C28" s="11" t="n"/>
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Sarafaz Khan</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="7" t="n"/>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Arjun Tendulkar</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="n"/>
-      <c r="B30" s="10" t="n"/>
-      <c r="C30" s="11" t="n"/>
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Ruturaj Gaikwad</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n"/>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="7" t="n"/>
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Romario Shepherd</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="n"/>
-      <c r="B32" s="10" t="n"/>
-      <c r="C32" s="11" t="n"/>
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Tom Latham</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n"/>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="7" t="n"/>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Shaheen Shah Afridi</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="n"/>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="11" t="n"/>
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Naseem Shah</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n"/>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="7" t="n"/>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Mohammad Amir</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="n"/>
-      <c r="B36" s="10" t="n"/>
-      <c r="C36" s="11" t="n"/>
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>Akhil</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>Chennai Super Kings</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n"/>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="7" t="n"/>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Devdutt Padikkal</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Kolkata Knight Riders</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="n"/>
-      <c r="B38" s="10" t="n"/>
-      <c r="C38" s="11" t="n"/>
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Vaibhav Suryavanshi</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Kolkata Knight Riders</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n"/>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="7" t="n"/>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Sikandar Raza</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Kolkata Knight Riders</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="n"/>
-      <c r="B40" s="10" t="n"/>
-      <c r="C40" s="11" t="n"/>
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Ashutosh Sharma</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>Kolkata Knight Riders</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n"/>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="7" t="n"/>
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Dharmendrasinh Jadeja</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Kolkata Knight Riders</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="n"/>
-      <c r="B42" s="10" t="n"/>
-      <c r="C42" s="11" t="n"/>
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Sameer Rizvi</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>Kolkata Knight Riders</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="n"/>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="7" t="n"/>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>T. Natarajan</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Kolkata Knight Riders</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="n"/>
-      <c r="B44" s="10" t="n"/>
-      <c r="C44" s="11" t="n"/>
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Umesh Yadav</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>Patna Panthers</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="n"/>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="7" t="n"/>
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Liam Livingstone</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Patna Panthers</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="n"/>
-      <c r="B46" s="10" t="n"/>
-      <c r="C46" s="11" t="n"/>
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Rahul Tripathi</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>Patna Panthers</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n"/>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="7" t="n"/>
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Suryakumar Yadav</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Patna Panthers</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="n"/>
-      <c r="B48" s="10" t="n"/>
-      <c r="C48" s="11" t="n"/>
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>Tim Seifert</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>Patna Panthers</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="n"/>
-      <c r="B49" s="6" t="n"/>
-      <c r="C49" s="7" t="n"/>
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Spencer Johnson</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Patna Panthers</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="9" t="n"/>
-      <c r="B50" s="10" t="n"/>
-      <c r="C50" s="11" t="n"/>
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Lhuan-dré Pretorius</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>Sunrisers Hydrabad</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n"/>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="7" t="n"/>
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>KL Rahul</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Sunrisers Hydrabad</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="n"/>
-      <c r="B52" s="10" t="n"/>
-      <c r="C52" s="11" t="n"/>
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>Angkrish Raghuvanshi</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>Sunrisers Hydrabad</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="n"/>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="7" t="n"/>
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Mohammed Siraj</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Sunrisers Hydrabad</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="9" t="n"/>
-      <c r="B54" s="10" t="n"/>
-      <c r="C54" s="11" t="n"/>
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>Baba Indrajith</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>Sunrisers Hydrabad</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="n"/>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="7" t="n"/>
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Nitish Rana</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Delhi Capitals</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="9" t="n"/>
-      <c r="B56" s="10" t="n"/>
-      <c r="C56" s="11" t="n"/>
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>Ben McKinney</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>Delhi Capitals</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="n"/>
-      <c r="B57" s="6" t="n"/>
-      <c r="C57" s="7" t="n"/>
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Keshav Maharaj</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Delhi Capitals</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="9" t="n"/>
-      <c r="B58" s="10" t="n"/>
-      <c r="C58" s="11" t="n"/>
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>Abrar Ahmed</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>Delhi Capitals</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="n"/>
-      <c r="B59" s="6" t="n"/>
-      <c r="C59" s="7" t="n"/>
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Faf Du Plesis</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Delhi Capitals</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="9" t="n"/>
-      <c r="B60" s="10" t="n"/>
-      <c r="C60" s="11" t="n"/>
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>Rajat Patidar</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>Delhi Capitals</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="n"/>
-      <c r="B61" s="6" t="n"/>
-      <c r="C61" s="7" t="n"/>
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Rinku Singh</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Gujarat Titans</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="9" t="n"/>
-      <c r="B62" s="10" t="n"/>
-      <c r="C62" s="11" t="n"/>
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>Sai Sudharsan</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Gujarat Titans</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="n"/>
-      <c r="B63" s="6" t="n"/>
-      <c r="C63" s="7" t="n"/>
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>Ishaan Kishaan</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Gujarat Titans</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="9" t="n"/>
-      <c r="B64" s="10" t="n"/>
-      <c r="C64" s="11" t="n"/>
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>Govinda Poddar</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>Gujarat Titans</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="n"/>
-      <c r="B65" s="6" t="n"/>
-      <c r="C65" s="7" t="n"/>
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Sanju Samson</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Lucknow Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="9" t="n"/>
-      <c r="B66" s="10" t="n"/>
-      <c r="C66" s="11" t="n"/>
+      <c r="A66" s="9" t="inlineStr">
+        <is>
+          <t>Dewald Brevis</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>Lucknow Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="n"/>
-      <c r="B67" s="6" t="n"/>
-      <c r="C67" s="7" t="n"/>
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Mayank Dagar</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Lucknow Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="9" t="n"/>
-      <c r="B68" s="10" t="n"/>
-      <c r="C68" s="11" t="n"/>
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>Abhishek Sharma</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>Lucknow Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="5" t="n"/>
-      <c r="B69" s="6" t="n"/>
-      <c r="C69" s="7" t="n"/>
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>Shaik Rasheed</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Imphal Igniter</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="9" t="n"/>
-      <c r="B70" s="10" t="n"/>
-      <c r="C70" s="11" t="n"/>
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>Chetan Sakariya</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>Imphal Igniter</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="n"/>
-      <c r="B71" s="6" t="n"/>
-      <c r="C71" s="7" t="n"/>
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>Quinton de Kock</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Imphal Igniter</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="9" t="n"/>
-      <c r="B72" s="10" t="n"/>
-      <c r="C72" s="11" t="n"/>
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>Joe Root</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>Imphal Igniter</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="n"/>
-      <c r="B73" s="6" t="n"/>
-      <c r="C73" s="7" t="n"/>
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Virat Kohli</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Imphal Igniter</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="9" t="n"/>
-      <c r="B74" s="10" t="n"/>
-      <c r="C74" s="11" t="n"/>
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>Vidwath Kaverappa</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>Imphal Igniter</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="n"/>
-      <c r="B75" s="6" t="n"/>
-      <c r="C75" s="7" t="n"/>
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>Siddharth Desai</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Imphal Igniter</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="9" t="n"/>
-      <c r="B76" s="10" t="n"/>
-      <c r="C76" s="11" t="n"/>
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>Ishant Sharma</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>Punjab Kings</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="n"/>
-      <c r="B77" s="6" t="n"/>
-      <c r="C77" s="7" t="n"/>
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>Deepak Hooda</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Punjab Kings</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="9" t="n"/>
-      <c r="B78" s="10" t="n"/>
-      <c r="C78" s="11" t="n"/>
+      <c r="A78" s="9" t="inlineStr">
+        <is>
+          <t>Sam Konstas</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>Punjab Kings</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="5" t="n"/>
-      <c r="B79" s="6" t="n"/>
-      <c r="C79" s="7" t="n"/>
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>Jitesh Sharma</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Punjab Kings</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="9" t="n"/>
-      <c r="B80" s="10" t="n"/>
-      <c r="C80" s="11" t="n"/>
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>Shubman Gill</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="C80" s="11" t="inlineStr">
+        <is>
+          <t>Punjab Kings</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="n"/>
-      <c r="B81" s="6" t="n"/>
-      <c r="C81" s="7" t="n"/>
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>Mitchell Starc</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Punjab Kings</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="9" t="n"/>
-      <c r="B82" s="10" t="n"/>
-      <c r="C82" s="11" t="n"/>
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>Jasprit Bumrah</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="n">
+        <v>24.25</v>
+      </c>
+      <c r="C82" s="11" t="inlineStr">
+        <is>
+          <t>Rising Pune Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="n"/>
-      <c r="B83" s="6" t="n"/>
-      <c r="C83" s="7" t="n"/>
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>Moeen Ali</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Rising Pune Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="9" t="n"/>
-      <c r="B84" s="10" t="n"/>
-      <c r="C84" s="11" t="n"/>
+      <c r="A84" s="9" t="inlineStr">
+        <is>
+          <t>Will Jacks</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="C84" s="11" t="inlineStr">
+        <is>
+          <t>Rising Pune Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="5" t="n"/>
-      <c r="B85" s="6" t="n"/>
-      <c r="C85" s="7" t="n"/>
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>Dasun Shanaka</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Rising Pune Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="9" t="n"/>
-      <c r="B86" s="10" t="n"/>
-      <c r="C86" s="11" t="n"/>
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>Amit Shukla</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="C86" s="11" t="inlineStr">
+        <is>
+          <t>Rising Pune Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="5" t="n"/>
-      <c r="B87" s="6" t="n"/>
-      <c r="C87" s="7" t="n"/>
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>Abhishek Powel</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Rising Pune Super Giants</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="9" t="n"/>
-      <c r="B88" s="10" t="n"/>
-      <c r="C88" s="11" t="n"/>
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>Harpreet Bhatia</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C88" s="11" t="inlineStr">
+        <is>
+          <t>Rajasthan Royals</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="n"/>
-      <c r="B89" s="6" t="n"/>
-      <c r="C89" s="7" t="n"/>
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>Musheer Khan</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>Rajasthan Royals</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="9" t="n"/>
-      <c r="B90" s="10" t="n"/>
-      <c r="C90" s="11" t="n"/>
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>Avesh Khan</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C90" s="11" t="inlineStr">
+        <is>
+          <t>Rajasthan Royals</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="n"/>
-      <c r="B91" s="6" t="n"/>
-      <c r="C91" s="7" t="n"/>
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>MS Dhoni</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Rajasthan Royals</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="9" t="n"/>
-      <c r="B92" s="10" t="n"/>
-      <c r="C92" s="11" t="n"/>
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>Glenn Maxwell</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C92" s="11" t="inlineStr">
+        <is>
+          <t>Rajasthan Royals</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="5" t="n"/>
-      <c r="B93" s="6" t="n"/>
-      <c r="C93" s="7" t="n"/>
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>Tom Bruce</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Rajasthan Royals</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="9" t="n"/>
-      <c r="B94" s="10" t="n"/>
-      <c r="C94" s="11" t="n"/>
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Harry Dixon</t>
+        </is>
+      </c>
+      <c r="B94" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C94" s="11" t="inlineStr">
+        <is>
+          <t>Rajasthan Royals</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="n"/>
-      <c r="B95" s="6" t="n"/>
-      <c r="C95" s="7" t="n"/>
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>Ajinkya Rahane</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Rajasthan Royals</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="9" t="n"/>
-      <c r="B96" s="10" t="n"/>
-      <c r="C96" s="11" t="n"/>
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>Priyansh Arya</t>
+        </is>
+      </c>
+      <c r="B96" s="10" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="C96" s="11" t="inlineStr">
+        <is>
+          <t>Rajasthan Royals</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="n"/>
-      <c r="B97" s="6" t="n"/>
-      <c r="C97" s="7" t="n"/>
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>Jason Holder</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>Kochi Tuskers</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="9" t="n"/>
-      <c r="B98" s="10" t="n"/>
-      <c r="C98" s="11" t="n"/>
+      <c r="A98" s="9" t="inlineStr">
+        <is>
+          <t>Kagiso Rabada</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="C98" s="11" t="inlineStr">
+        <is>
+          <t>Kochi Tuskers</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="n"/>
-      <c r="B99" s="6" t="n"/>
-      <c r="C99" s="7" t="n"/>
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>Heinrich Klassen</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>Kochi Tuskers</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="9" t="n"/>
-      <c r="B100" s="10" t="n"/>
-      <c r="C100" s="11" t="n"/>
+      <c r="A100" s="9" t="inlineStr">
+        <is>
+          <t>Nikhil Gangta</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C100" s="11" t="inlineStr">
+        <is>
+          <t>Kochi Tuskers</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="n"/>
-      <c r="B101" s="6" t="n"/>
-      <c r="C101" s="7" t="n"/>
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Hardik Pandya</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>Guwahati Chargers</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="9" t="n"/>
-      <c r="B102" s="10" t="n"/>
-      <c r="C102" s="11" t="n"/>
+      <c r="A102" s="9" t="inlineStr">
+        <is>
+          <t>Shakib Al Hasan</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C102" s="11" t="inlineStr">
+        <is>
+          <t>Guwahati Chargers</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="n"/>
-      <c r="B103" s="6" t="n"/>
-      <c r="C103" s="7" t="n"/>
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>Nehal Wadhera</t>
+        </is>
+      </c>
+      <c r="B103" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>Guwahati Chargers</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="9" t="n"/>
-      <c r="B104" s="10" t="n"/>
-      <c r="C104" s="11" t="n"/>
+      <c r="A104" s="9" t="inlineStr">
+        <is>
+          <t>Rishabh Pant</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C104" s="11" t="inlineStr">
+        <is>
+          <t>Guwahati Chargers</t>
+        </is>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="n"/>
-      <c r="B105" s="6" t="n"/>
-      <c r="C105" s="7" t="n"/>
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>Wiaan Mulder</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>Guwahati Chargers</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="9" t="n"/>
-      <c r="B106" s="10" t="n"/>
-      <c r="C106" s="11" t="n"/>
+      <c r="A106" s="9" t="inlineStr">
+        <is>
+          <t>Maheesh Theekshana</t>
+        </is>
+      </c>
+      <c r="B106" s="10" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="C106" s="11" t="inlineStr">
+        <is>
+          <t>Guwahati Chargers</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n"/>
@@ -9596,7 +10566,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>Mumbai Indians</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
@@ -9618,7 +10588,7 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>Royal Challangers Banglore</t>
         </is>
       </c>
       <c r="B5" s="10" t="n">
@@ -9640,7 +10610,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Team 3</t>
+          <t>Chennai Super Kings</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -9662,7 +10632,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Team 4</t>
+          <t>Kolkata Knight Riders</t>
         </is>
       </c>
       <c r="B7" s="10" t="n">
@@ -9684,7 +10654,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Team 5</t>
+          <t>Patna Panthers</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
@@ -9706,7 +10676,7 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Team 6</t>
+          <t>Sunrisers Hydrabad</t>
         </is>
       </c>
       <c r="B9" s="10" t="n">
@@ -9728,7 +10698,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Team 7</t>
+          <t>Delhi Capitals</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
@@ -9750,7 +10720,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Team 8</t>
+          <t>Gujarat Titans</t>
         </is>
       </c>
       <c r="B11" s="10" t="n">
@@ -9772,7 +10742,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Team 9</t>
+          <t>Lucknow Super Giants</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
@@ -9794,7 +10764,7 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Team 10</t>
+          <t>Imphal Igniter</t>
         </is>
       </c>
       <c r="B13" s="10" t="n">
@@ -9816,7 +10786,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Team 11</t>
+          <t>Punjab Kings</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
@@ -9838,7 +10808,7 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Team 12</t>
+          <t>Rising Pune Super Giants</t>
         </is>
       </c>
       <c r="B15" s="10" t="n">
@@ -9860,7 +10830,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Team 13</t>
+          <t>Rajasthan Royals</t>
         </is>
       </c>
       <c r="B16" s="6" t="n">
@@ -9882,7 +10852,7 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Team 14</t>
+          <t>Kochi Tuskers</t>
         </is>
       </c>
       <c r="B17" s="10" t="n">
@@ -9904,7 +10874,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Team 15</t>
+          <t>Guwahati Chargers</t>
         </is>
       </c>
       <c r="B18" s="6" t="n">

</xml_diff>